<commit_message>
Added comments to gui and matchmaking project trackers
</commit_message>
<xml_diff>
--- a/Iteration_2/Echo_Review/Echo/project_tracker_gui.xlsx
+++ b/Iteration_2/Echo_Review/Echo/project_tracker_gui.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E42492D4-A913-4DA0-A5BF-2FD5969FDFC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067A9D08-FFC3-41D3-B54A-AF9DE92689C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project tracker" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,6 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Project tracker'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,6 +35,60 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={787986D8-1FDC-469D-A088-8C0F63DA9C53}</author>
+    <author>tc={AE9EA276-0B44-4276-A3F9-7772F2345B51}</author>
+    <author>tc={ED8FB9F1-6DAA-4E83-86C1-DB279CE5868C}</author>
+    <author>tc={556FE37B-62A8-443B-B67B-433C0E7A5AB4}</author>
+    <author>tc={97438B52-7420-4EFC-976B-B339DA82ACC9}</author>
+  </authors>
+  <commentList>
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{787986D8-1FDC-469D-A088-8C0F63DA9C53}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assigning all the planning to one student/group and all the coding to another is not a great idea because there won’t be someone with a great understanding of the plan working on and overlooking the coding process who can ensure that it accurately follows the initial plan. i.e there won’t be great communication and coordination between the coding and planning sides of the project, hence greater chance for errors, problems, and poorly structured code later on</t>
+      </text>
+    </comment>
+    <comment ref="M5" authorId="1" shapeId="0" xr:uid="{AE9EA276-0B44-4276-A3F9-7772F2345B51}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Student 6 could add a bit of detail to the task notes, better describing the work they did. Ex what use case description did they finish, what did they add to the diagrams to finish them, what classes/functions are the descriptions and diagrams for, etc</t>
+      </text>
+    </comment>
+    <comment ref="H6" authorId="2" shapeId="0" xr:uid="{ED8FB9F1-6DAA-4E83-86C1-DB279CE5868C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    The estimated duration in days for tasks 2-6 suggest that they are rather large and would probably be able to be split among multiple individuals rather than just Student 5 and 6. i.e It would’ve been a good idea to split these tasks among more people</t>
+      </text>
+    </comment>
+    <comment ref="K7" authorId="3" shapeId="0" xr:uid="{556FE37B-62A8-443B-B67B-433C0E7A5AB4}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Certain tasks get finished within 1-4 hours of work but is spread out between several weeks. This is very strange, and the students who did these tasks should clarify the low work hours compared to long duration in days. It could be caused by other matters delaying the task’s completion, omitting work time from the actual work hours (for whatever reason), or a sign of bad work ethic/inefficient work. In summary, clarification regarding this strange work duration should be provided</t>
+      </text>
+    </comment>
+    <comment ref="M9" authorId="4" shapeId="0" xr:uid="{97438B52-7420-4EFC-976B-B339DA82ACC9}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Student 5’s task notes imply that they did not finish the tasks and are actively working on them. Either change the wording, or don’t list them as completed.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="49">
   <si>
@@ -196,7 +249,7 @@
     <numFmt numFmtId="164" formatCode="&quot;Over/Under flag&quot;;&quot;&quot;;&quot;&quot;"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="3" tint="-0.499984740745262"/>
@@ -350,6 +403,12 @@
       <color theme="9" tint="-0.499984740745262"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="8">
@@ -1240,6 +1299,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProjectTracker" displayName="ProjectTracker" ref="B4:M12" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="B4:M12" xr:uid="{00000000-0009-0000-0100-000001000000}">
@@ -1527,26 +1590,46 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="D5" dT="2024-11-12T23:50:26.37" personId="{00000000-0000-0000-0000-000000000000}" id="{787986D8-1FDC-469D-A088-8C0F63DA9C53}">
+    <text>Assigning all the planning to one student/group and all the coding to another is not a great idea because there won’t be someone with a great understanding of the plan working on and overlooking the coding process who can ensure that it accurately follows the initial plan. i.e there won’t be great communication and coordination between the coding and planning sides of the project, hence greater chance for errors, problems, and poorly structured code later on</text>
+  </threadedComment>
+  <threadedComment ref="M5" dT="2024-11-13T04:01:32.97" personId="{00000000-0000-0000-0000-000000000000}" id="{AE9EA276-0B44-4276-A3F9-7772F2345B51}">
+    <text>Student 6 could add a bit of detail to the task notes, better describing the work they did. Ex what use case description did they finish, what did they add to the diagrams to finish them, what classes/functions are the descriptions and diagrams for, etc</text>
+  </threadedComment>
+  <threadedComment ref="H6" dT="2024-11-13T01:47:36.32" personId="{00000000-0000-0000-0000-000000000000}" id="{ED8FB9F1-6DAA-4E83-86C1-DB279CE5868C}">
+    <text>The estimated duration in days for tasks 2-6 suggest that they are rather large and would probably be able to be split among multiple individuals rather than just Student 5 and 6. i.e It would’ve been a good idea to split these tasks among more people</text>
+  </threadedComment>
+  <threadedComment ref="K7" dT="2024-11-12T23:58:51.82" personId="{00000000-0000-0000-0000-000000000000}" id="{556FE37B-62A8-443B-B67B-433C0E7A5AB4}">
+    <text>Certain tasks get finished within 1-4 hours of work but is spread out between several weeks. This is very strange, and the students who did these tasks should clarify the low work hours compared to long duration in days. It could be caused by other matters delaying the task’s completion, omitting work time from the actual work hours (for whatever reason), or a sign of bad work ethic/inefficient work. In summary, clarification regarding this strange work duration should be provided</text>
+  </threadedComment>
+  <threadedComment ref="M9" dT="2024-11-13T04:03:22.75" personId="{00000000-0000-0000-0000-000000000000}" id="{97438B52-7420-4EFC-976B-B339DA82ACC9}">
+    <text>Student 5’s task notes imply that they did not finish the tasks and are actively working on them. Either change the wording, or don’t list them as completed.</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1">
     <tabColor theme="6"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N12"/>
-  <sheetFormatPr defaultColWidth="9.0703125" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" style="3" customWidth="1"/>
-    <col min="2" max="4" width="18.7109375" style="19" customWidth="1"/>
-    <col min="5" max="6" width="18.7109375" style="20" customWidth="1"/>
-    <col min="7" max="8" width="18.7109375" style="19" customWidth="1"/>
-    <col min="9" max="10" width="16.78515625" style="20" customWidth="1"/>
+    <col min="1" max="1" width="6.7265625" style="3" customWidth="1"/>
+    <col min="2" max="4" width="18.7265625" style="19" customWidth="1"/>
+    <col min="5" max="6" width="18.7265625" style="20" customWidth="1"/>
+    <col min="7" max="8" width="18.7265625" style="19" customWidth="1"/>
+    <col min="9" max="10" width="16.81640625" style="20" customWidth="1"/>
     <col min="11" max="12" width="16" style="19" customWidth="1"/>
-    <col min="13" max="13" width="20.35546875" style="19" customWidth="1"/>
-    <col min="14" max="14" width="6.7109375" style="3" customWidth="1"/>
-    <col min="15" max="15" width="4.2109375" style="2" customWidth="1"/>
-    <col min="16" max="40" width="3.28515625" style="2" customWidth="1"/>
-    <col min="41" max="16384" width="9.0703125" style="2"/>
+    <col min="13" max="13" width="20.36328125" style="19" customWidth="1"/>
+    <col min="14" max="14" width="6.7265625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="4.1796875" style="2" customWidth="1"/>
+    <col min="16" max="40" width="3.26953125" style="2" customWidth="1"/>
+    <col min="41" max="16384" width="9.08984375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1565,7 +1648,7 @@
       <c r="M1" s="3"/>
       <c r="N1" s="3"/>
     </row>
-    <row r="2" spans="1:14" s="5" customFormat="1" ht="80.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" s="5" customFormat="1" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="26" t="s">
         <v>22</v>
@@ -1603,7 +1686,7 @@
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
     </row>
-    <row r="4" spans="1:14" s="5" customFormat="1" ht="62.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" s="5" customFormat="1" ht="62.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11"/>
       <c r="B4" s="17" t="s">
         <v>18</v>
@@ -1656,11 +1739,11 @@
       </c>
       <c r="E5" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45596</v>
+        <v>45603</v>
       </c>
       <c r="F5" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45608</v>
       </c>
       <c r="G5" s="18">
         <v>10</v>
@@ -1671,11 +1754,11 @@
       </c>
       <c r="I5" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45596</v>
+        <v>45603</v>
       </c>
       <c r="J5" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45608</v>
       </c>
       <c r="K5" s="18">
         <v>5</v>
@@ -1702,11 +1785,11 @@
       </c>
       <c r="E6" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45596</v>
+        <v>45603</v>
       </c>
       <c r="F6" s="25">
         <f ca="1">TODAY()+5</f>
-        <v>45606</v>
+        <v>45613</v>
       </c>
       <c r="G6" s="18">
         <v>4</v>
@@ -1717,11 +1800,11 @@
       </c>
       <c r="I6" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45596</v>
+        <v>45603</v>
       </c>
       <c r="J6" s="25">
         <f ca="1">TODAY()+5</f>
-        <v>45606</v>
+        <v>45613</v>
       </c>
       <c r="K6" s="18">
         <v>6</v>
@@ -1748,11 +1831,11 @@
       </c>
       <c r="E7" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45608</v>
       </c>
       <c r="F7" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45625</v>
       </c>
       <c r="G7" s="18">
         <v>50</v>
@@ -1763,11 +1846,11 @@
       </c>
       <c r="I7" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45608</v>
       </c>
       <c r="J7" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45625</v>
       </c>
       <c r="K7" s="18">
         <v>4</v>
@@ -1794,11 +1877,11 @@
       </c>
       <c r="E8" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45608</v>
       </c>
       <c r="F8" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45625</v>
       </c>
       <c r="G8" s="18">
         <v>15</v>
@@ -1809,11 +1892,11 @@
       </c>
       <c r="I8" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45608</v>
       </c>
       <c r="J8" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45625</v>
       </c>
       <c r="K8" s="18">
         <v>1</v>
@@ -1840,11 +1923,11 @@
       </c>
       <c r="E9" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45608</v>
       </c>
       <c r="F9" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45625</v>
       </c>
       <c r="G9" s="18">
         <v>10</v>
@@ -1855,11 +1938,11 @@
       </c>
       <c r="I9" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45608</v>
       </c>
       <c r="J9" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45625</v>
       </c>
       <c r="K9" s="18">
         <v>1</v>
@@ -1886,11 +1969,11 @@
       </c>
       <c r="E10" s="25">
         <f ca="1">TODAY()+3</f>
-        <v>45604</v>
+        <v>45611</v>
       </c>
       <c r="F10" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45625</v>
       </c>
       <c r="G10" s="18">
         <v>5</v>
@@ -1901,11 +1984,11 @@
       </c>
       <c r="I10" s="25">
         <f ca="1">TODAY()+3</f>
-        <v>45604</v>
+        <v>45611</v>
       </c>
       <c r="J10" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45625</v>
       </c>
       <c r="K10" s="18">
         <v>6</v>
@@ -1996,8 +2079,9 @@
   <pageSetup fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter differentFirst="1"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2005,12 +2089,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C52F64F2-A0CB-432E-B537-8AB164D6506B}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" style="27" customWidth="1"/>
-    <col min="2" max="2" width="20.0703125" style="27" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" style="27" customWidth="1"/>
-    <col min="4" max="16384" width="8.7109375" style="27"/>
+    <col min="1" max="1" width="12.7265625" style="27" customWidth="1"/>
+    <col min="2" max="2" width="20.08984375" style="27" customWidth="1"/>
+    <col min="3" max="3" width="16.7265625" style="27" customWidth="1"/>
+    <col min="4" max="16384" width="8.7265625" style="27"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2057,9 +2141,9 @@
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" style="12" customWidth="1"/>
-    <col min="2" max="3" width="18.42578125" style="23" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" style="13" customWidth="1"/>
+    <col min="1" max="1" width="6.7265625" style="12" customWidth="1"/>
+    <col min="2" max="3" width="18.453125" style="23" customWidth="1"/>
+    <col min="4" max="4" width="6.7265625" style="13" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -2069,7 +2153,7 @@
       <c r="C1" s="12"/>
       <c r="D1" s="12"/>
     </row>
-    <row r="2" spans="1:4" customFormat="1" ht="80.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" customFormat="1" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12"/>
       <c r="B2" s="16" t="s">
         <v>4</v>
@@ -2083,7 +2167,7 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4" customFormat="1" ht="62.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" customFormat="1" ht="62.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14"/>
       <c r="B4" s="22" t="s">
         <v>5</v>
@@ -2175,23 +2259,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2507,22 +2580,29 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9066C173-72E5-4455-ACFB-9A7596D30A2B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{648F31BC-5AA3-42BF-80F4-A797E59C4FBD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2549,9 +2629,13 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{648F31BC-5AA3-42BF-80F4-A797E59C4FBD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9066C173-72E5-4455-ACFB-9A7596D30A2B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Adjusted comments and added a few more
</commit_message>
<xml_diff>
--- a/Iteration_2/Echo_Review/Echo/project_tracker_gui.xlsx
+++ b/Iteration_2/Echo_Review/Echo/project_tracker_gui.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067A9D08-FFC3-41D3-B54A-AF9DE92689C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A523674B-FEC9-41FF-8AFB-D3A1D435E527}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,6 +42,7 @@
     <author>tc={AE9EA276-0B44-4276-A3F9-7772F2345B51}</author>
     <author>tc={ED8FB9F1-6DAA-4E83-86C1-DB279CE5868C}</author>
     <author>tc={556FE37B-62A8-443B-B67B-433C0E7A5AB4}</author>
+    <author>tc={2BA0C9CA-C6B8-4B33-9AAD-493E02C58D14}</author>
     <author>tc={97438B52-7420-4EFC-976B-B339DA82ACC9}</author>
   </authors>
   <commentList>
@@ -66,7 +67,7 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    The estimated duration in days for tasks 2-6 suggest that they are rather large and would probably be able to be split among multiple individuals rather than just Student 5 and 6. i.e It would’ve been a good idea to split these tasks among more people</t>
+    The estimated duration in days and hours for tasks 2-6 suggest that they are rather large and would probably be able to be split among multiple individuals rather than just Student 5 and 6. i.e It would’ve been a good idea to split these tasks among more people</t>
       </text>
     </comment>
     <comment ref="K7" authorId="3" shapeId="0" xr:uid="{556FE37B-62A8-443B-B67B-433C0E7A5AB4}">
@@ -77,7 +78,15 @@
     Certain tasks get finished within 1-4 hours of work but is spread out between several weeks. This is very strange, and the students who did these tasks should clarify the low work hours compared to long duration in days. It could be caused by other matters delaying the task’s completion, omitting work time from the actual work hours (for whatever reason), or a sign of bad work ethic/inefficient work. In summary, clarification regarding this strange work duration should be provided</t>
       </text>
     </comment>
-    <comment ref="M9" authorId="4" shapeId="0" xr:uid="{97438B52-7420-4EFC-976B-B339DA82ACC9}">
+    <comment ref="B8" authorId="4" shapeId="0" xr:uid="{2BA0C9CA-C6B8-4B33-9AAD-493E02C58D14}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Student 5’s tasks don’t really reflect the work described on the task notes. It would be better to separate the unrelated work and list it as a separate task for better documentation, and mention the work related most to the task in the notes</t>
+      </text>
+    </comment>
+    <comment ref="M9" authorId="5" shapeId="0" xr:uid="{97438B52-7420-4EFC-976B-B339DA82ACC9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1599,10 +1608,13 @@
     <text>Student 6 could add a bit of detail to the task notes, better describing the work they did. Ex what use case description did they finish, what did they add to the diagrams to finish them, what classes/functions are the descriptions and diagrams for, etc</text>
   </threadedComment>
   <threadedComment ref="H6" dT="2024-11-13T01:47:36.32" personId="{00000000-0000-0000-0000-000000000000}" id="{ED8FB9F1-6DAA-4E83-86C1-DB279CE5868C}">
-    <text>The estimated duration in days for tasks 2-6 suggest that they are rather large and would probably be able to be split among multiple individuals rather than just Student 5 and 6. i.e It would’ve been a good idea to split these tasks among more people</text>
+    <text>The estimated duration in days and hours for tasks 2-6 suggest that they are rather large and would probably be able to be split among multiple individuals rather than just Student 5 and 6. i.e It would’ve been a good idea to split these tasks among more people</text>
   </threadedComment>
   <threadedComment ref="K7" dT="2024-11-12T23:58:51.82" personId="{00000000-0000-0000-0000-000000000000}" id="{556FE37B-62A8-443B-B67B-433C0E7A5AB4}">
     <text>Certain tasks get finished within 1-4 hours of work but is spread out between several weeks. This is very strange, and the students who did these tasks should clarify the low work hours compared to long duration in days. It could be caused by other matters delaying the task’s completion, omitting work time from the actual work hours (for whatever reason), or a sign of bad work ethic/inefficient work. In summary, clarification regarding this strange work duration should be provided</text>
+  </threadedComment>
+  <threadedComment ref="B8" dT="2024-11-14T03:11:18.47" personId="{00000000-0000-0000-0000-000000000000}" id="{2BA0C9CA-C6B8-4B33-9AAD-493E02C58D14}">
+    <text>Student 5’s tasks don’t really reflect the work described on the task notes. It would be better to separate the unrelated work and list it as a separate task for better documentation, and mention the work related most to the task in the notes</text>
   </threadedComment>
   <threadedComment ref="M9" dT="2024-11-13T04:03:22.75" personId="{00000000-0000-0000-0000-000000000000}" id="{97438B52-7420-4EFC-976B-B339DA82ACC9}">
     <text>Student 5’s task notes imply that they did not finish the tasks and are actively working on them. Either change the wording, or don’t list them as completed.</text>
@@ -1739,11 +1751,11 @@
       </c>
       <c r="E5" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45603</v>
+        <v>45604</v>
       </c>
       <c r="F5" s="25">
         <f ca="1">TODAY()</f>
-        <v>45608</v>
+        <v>45609</v>
       </c>
       <c r="G5" s="18">
         <v>10</v>
@@ -1754,11 +1766,11 @@
       </c>
       <c r="I5" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45603</v>
+        <v>45604</v>
       </c>
       <c r="J5" s="25">
         <f ca="1">TODAY()</f>
-        <v>45608</v>
+        <v>45609</v>
       </c>
       <c r="K5" s="18">
         <v>5</v>
@@ -1785,11 +1797,11 @@
       </c>
       <c r="E6" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45603</v>
+        <v>45604</v>
       </c>
       <c r="F6" s="25">
         <f ca="1">TODAY()+5</f>
-        <v>45613</v>
+        <v>45614</v>
       </c>
       <c r="G6" s="18">
         <v>4</v>
@@ -1800,11 +1812,11 @@
       </c>
       <c r="I6" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45603</v>
+        <v>45604</v>
       </c>
       <c r="J6" s="25">
         <f ca="1">TODAY()+5</f>
-        <v>45613</v>
+        <v>45614</v>
       </c>
       <c r="K6" s="18">
         <v>6</v>
@@ -1831,11 +1843,11 @@
       </c>
       <c r="E7" s="25">
         <f ca="1">TODAY()</f>
-        <v>45608</v>
+        <v>45609</v>
       </c>
       <c r="F7" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45625</v>
+        <v>45626</v>
       </c>
       <c r="G7" s="18">
         <v>50</v>
@@ -1846,11 +1858,11 @@
       </c>
       <c r="I7" s="25">
         <f ca="1">TODAY()</f>
-        <v>45608</v>
+        <v>45609</v>
       </c>
       <c r="J7" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45625</v>
+        <v>45626</v>
       </c>
       <c r="K7" s="18">
         <v>4</v>
@@ -1877,11 +1889,11 @@
       </c>
       <c r="E8" s="25">
         <f ca="1">TODAY()</f>
-        <v>45608</v>
+        <v>45609</v>
       </c>
       <c r="F8" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45625</v>
+        <v>45626</v>
       </c>
       <c r="G8" s="18">
         <v>15</v>
@@ -1892,11 +1904,11 @@
       </c>
       <c r="I8" s="25">
         <f ca="1">TODAY()</f>
-        <v>45608</v>
+        <v>45609</v>
       </c>
       <c r="J8" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45625</v>
+        <v>45626</v>
       </c>
       <c r="K8" s="18">
         <v>1</v>
@@ -1923,11 +1935,11 @@
       </c>
       <c r="E9" s="25">
         <f ca="1">TODAY()</f>
-        <v>45608</v>
+        <v>45609</v>
       </c>
       <c r="F9" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45625</v>
+        <v>45626</v>
       </c>
       <c r="G9" s="18">
         <v>10</v>
@@ -1938,11 +1950,11 @@
       </c>
       <c r="I9" s="25">
         <f ca="1">TODAY()</f>
-        <v>45608</v>
+        <v>45609</v>
       </c>
       <c r="J9" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45625</v>
+        <v>45626</v>
       </c>
       <c r="K9" s="18">
         <v>1</v>
@@ -1969,11 +1981,11 @@
       </c>
       <c r="E10" s="25">
         <f ca="1">TODAY()+3</f>
-        <v>45611</v>
+        <v>45612</v>
       </c>
       <c r="F10" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45625</v>
+        <v>45626</v>
       </c>
       <c r="G10" s="18">
         <v>5</v>
@@ -1984,11 +1996,11 @@
       </c>
       <c r="I10" s="25">
         <f ca="1">TODAY()+3</f>
-        <v>45611</v>
+        <v>45612</v>
       </c>
       <c r="J10" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45625</v>
+        <v>45626</v>
       </c>
       <c r="K10" s="18">
         <v>6</v>

</xml_diff>

<commit_message>
Echo: gui and matchmaking leaderboard project trackers
</commit_message>
<xml_diff>
--- a/Iteration_2/Echo_Review/Echo/project_tracker_gui.xlsx
+++ b/Iteration_2/Echo_Review/Echo/project_tracker_gui.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28129"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E42492D4-A913-4DA0-A5BF-2FD5969FDFC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A85D225B-61FB-4CE6-925D-EE0F38C3685B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project tracker" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,6 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Project tracker'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,6 +33,105 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={787986D8-1FDC-469D-A088-8C0F63DA9C53}</author>
+    <author>tc={AE9EA276-0B44-4276-A3F9-7772F2345B51}</author>
+    <author>tc={ED8FB9F1-6DAA-4E83-86C1-DB279CE5868C}</author>
+    <author>tc={556FE37B-62A8-443B-B67B-433C0E7A5AB4}</author>
+    <author>tc={2BA0C9CA-C6B8-4B33-9AAD-493E02C58D14}</author>
+    <author>tc={97438B52-7420-4EFC-976B-B339DA82ACC9}</author>
+  </authors>
+  <commentList>
+    <comment ref="D5" authorId="0" shapeId="0" xr:uid="{787986D8-1FDC-469D-A088-8C0F63DA9C53}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Assigning all the planning to one student/group and all the coding to another is not a great idea because there won’t be someone with a great understanding of the plan working on and overlooking the coding process who can ensure that it accurately follows the initial plan. i.e there won’t be great communication and coordination between the coding and planning sides of the project, hence greater chance for errors, problems, and poorly structured code later on</t>
+      </text>
+    </comment>
+    <comment ref="M5" authorId="1" shapeId="0" xr:uid="{AE9EA276-0B44-4276-A3F9-7772F2345B51}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Student 6 could add a bit of detail to the task notes, better describing the work they did. Ex which use case description did they finish, what did they add to the diagrams in order to finish them, what classes/functions are the descriptions and diagrams for, etc</t>
+      </text>
+    </comment>
+    <comment ref="H6" authorId="2" shapeId="0" xr:uid="{ED8FB9F1-6DAA-4E83-86C1-DB279CE5868C}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    The estimated duration in days and hours for tasks 2-6 suggest that they are rather large and would probably be able to be split among multiple individuals rather than just Student 5 and 6. i.e It might’ve been a good idea to split these tasks among more people if possible</t>
+      </text>
+    </comment>
+    <comment ref="K7" authorId="3" shapeId="0" xr:uid="{556FE37B-62A8-443B-B67B-433C0E7A5AB4}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Certain tasks get finished within 1-4 hours of work but is spread out between several weeks. This is very strange, and the students who did these tasks should clarify the low work hours compared to long duration in days. If the issue is simply neglecting to record the actual days taken and simply copy/pasting the estimated duration, then it should simply be changed to reflect the actual time taken.</t>
+      </text>
+    </comment>
+    <comment ref="B8" authorId="4" shapeId="0" xr:uid="{2BA0C9CA-C6B8-4B33-9AAD-493E02C58D14}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Student 5’s tasks don’t seem to reflect the work described on the task notes. It would be better to separate the unrelated work and list it as a separate task for better documentation, and mention the work related most to the task in the notes; or to reword the task notes to better match the task</t>
+      </text>
+    </comment>
+    <comment ref="M9" authorId="5" shapeId="0" xr:uid="{97438B52-7420-4EFC-976B-B339DA82ACC9}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Student 5’s task notes imply that they did not finish the tasks and are actively working on them. Either change the wording, or don’t list them as completed.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={8E089076-CF64-4085-B660-1C306875BDD2}</author>
+  </authors>
+  <commentList>
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{8E089076-CF64-4085-B660-1C306875BDD2}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Task lookup page incomplete</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={69215A04-AE1B-4A3B-ADD1-E683A6B27986}</author>
+  </authors>
+  <commentList>
+    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{69215A04-AE1B-4A3B-ADD1-E683A6B27986}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    No students were named and no tasks regarding design were done. Not necessarily a bad thing but if there were no tasks related to design to begin with, it maybe shouldn’t be listed as a category here</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1240,6 +1338,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ProjectTracker" displayName="ProjectTracker" ref="B4:M12" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
   <autoFilter ref="B4:M12" xr:uid="{00000000-0009-0000-0100-000001000000}">
@@ -1527,26 +1629,65 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="D5" dT="2024-11-12T23:50:26.37" personId="{00000000-0000-0000-0000-000000000000}" id="{787986D8-1FDC-469D-A088-8C0F63DA9C53}">
+    <text>Assigning all the planning to one student/group and all the coding to another is not a great idea because there won’t be someone with a great understanding of the plan working on and overlooking the coding process who can ensure that it accurately follows the initial plan. i.e there won’t be great communication and coordination between the coding and planning sides of the project, hence greater chance for errors, problems, and poorly structured code later on</text>
+  </threadedComment>
+  <threadedComment ref="M5" dT="2024-11-13T04:01:32.97" personId="{00000000-0000-0000-0000-000000000000}" id="{AE9EA276-0B44-4276-A3F9-7772F2345B51}">
+    <text>Student 6 could add a bit of detail to the task notes, better describing the work they did. Ex which use case description did they finish, what did they add to the diagrams in order to finish them, what classes/functions are the descriptions and diagrams for, etc</text>
+  </threadedComment>
+  <threadedComment ref="H6" dT="2024-11-13T01:47:36.32" personId="{00000000-0000-0000-0000-000000000000}" id="{ED8FB9F1-6DAA-4E83-86C1-DB279CE5868C}">
+    <text>The estimated duration in days and hours for tasks 2-6 suggest that they are rather large and would probably be able to be split among multiple individuals rather than just Student 5 and 6. i.e It might’ve been a good idea to split these tasks among more people if possible</text>
+  </threadedComment>
+  <threadedComment ref="K7" dT="2024-11-12T23:58:51.82" personId="{00000000-0000-0000-0000-000000000000}" id="{556FE37B-62A8-443B-B67B-433C0E7A5AB4}">
+    <text>Certain tasks get finished within 1-4 hours of work but is spread out between several weeks. This is very strange, and the students who did these tasks should clarify the low work hours compared to long duration in days. If the issue is simply neglecting to record the actual days taken and simply copy/pasting the estimated duration, then it should simply be changed to reflect the actual time taken.</text>
+  </threadedComment>
+  <threadedComment ref="B8" dT="2024-11-14T03:11:18.47" personId="{00000000-0000-0000-0000-000000000000}" id="{2BA0C9CA-C6B8-4B33-9AAD-493E02C58D14}">
+    <text>Student 5’s tasks don’t seem to reflect the work described on the task notes. It would be better to separate the unrelated work and list it as a separate task for better documentation, and mention the work related most to the task in the notes; or to reword the task notes to better match the task</text>
+  </threadedComment>
+  <threadedComment ref="M9" dT="2024-11-13T04:03:22.75" personId="{00000000-0000-0000-0000-000000000000}" id="{97438B52-7420-4EFC-976B-B339DA82ACC9}">
+    <text>Student 5’s task notes imply that they did not finish the tasks and are actively working on them. Either change the wording, or don’t list them as completed.</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="D1" dT="2024-11-14T04:22:12.21" personId="{00000000-0000-0000-0000-000000000000}" id="{8E089076-CF64-4085-B660-1C306875BDD2}">
+    <text>Task lookup page incomplete</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="C5" dT="2024-11-14T04:20:54.84" personId="{00000000-0000-0000-0000-000000000000}" id="{69215A04-AE1B-4A3B-ADD1-E683A6B27986}">
+    <text>No students were named and no tasks regarding design were done. Not necessarily a bad thing but if there were no tasks related to design to begin with, it maybe shouldn’t be listed as a category here</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1">
     <tabColor theme="6"/>
     <pageSetUpPr autoPageBreaks="0" fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:N12"/>
-  <sheetFormatPr defaultColWidth="9.0703125" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.08984375" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" style="3" customWidth="1"/>
-    <col min="2" max="4" width="18.7109375" style="19" customWidth="1"/>
-    <col min="5" max="6" width="18.7109375" style="20" customWidth="1"/>
-    <col min="7" max="8" width="18.7109375" style="19" customWidth="1"/>
-    <col min="9" max="10" width="16.78515625" style="20" customWidth="1"/>
+    <col min="1" max="1" width="6.7265625" style="3" customWidth="1"/>
+    <col min="2" max="4" width="18.7265625" style="19" customWidth="1"/>
+    <col min="5" max="6" width="18.7265625" style="20" customWidth="1"/>
+    <col min="7" max="8" width="18.7265625" style="19" customWidth="1"/>
+    <col min="9" max="10" width="16.81640625" style="20" customWidth="1"/>
     <col min="11" max="12" width="16" style="19" customWidth="1"/>
-    <col min="13" max="13" width="20.35546875" style="19" customWidth="1"/>
-    <col min="14" max="14" width="6.7109375" style="3" customWidth="1"/>
-    <col min="15" max="15" width="4.2109375" style="2" customWidth="1"/>
-    <col min="16" max="40" width="3.28515625" style="2" customWidth="1"/>
-    <col min="41" max="16384" width="9.0703125" style="2"/>
+    <col min="13" max="13" width="20.36328125" style="19" customWidth="1"/>
+    <col min="14" max="14" width="6.7265625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="4.1796875" style="2" customWidth="1"/>
+    <col min="16" max="40" width="3.26953125" style="2" customWidth="1"/>
+    <col min="41" max="16384" width="9.08984375" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" s="5" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1565,7 +1706,7 @@
       <c r="M1" s="3"/>
       <c r="N1" s="3"/>
     </row>
-    <row r="2" spans="1:14" s="5" customFormat="1" ht="80.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" s="5" customFormat="1" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3"/>
       <c r="B2" s="26" t="s">
         <v>22</v>
@@ -1603,7 +1744,7 @@
       <c r="M3" s="3"/>
       <c r="N3" s="3"/>
     </row>
-    <row r="4" spans="1:14" s="5" customFormat="1" ht="62.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" s="5" customFormat="1" ht="62.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11"/>
       <c r="B4" s="17" t="s">
         <v>18</v>
@@ -1656,11 +1797,11 @@
       </c>
       <c r="E5" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45596</v>
+        <v>45604</v>
       </c>
       <c r="F5" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45609</v>
       </c>
       <c r="G5" s="18">
         <v>10</v>
@@ -1671,11 +1812,11 @@
       </c>
       <c r="I5" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45596</v>
+        <v>45604</v>
       </c>
       <c r="J5" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45609</v>
       </c>
       <c r="K5" s="18">
         <v>5</v>
@@ -1702,11 +1843,11 @@
       </c>
       <c r="E6" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45596</v>
+        <v>45604</v>
       </c>
       <c r="F6" s="25">
         <f ca="1">TODAY()+5</f>
-        <v>45606</v>
+        <v>45614</v>
       </c>
       <c r="G6" s="18">
         <v>4</v>
@@ -1717,11 +1858,11 @@
       </c>
       <c r="I6" s="25">
         <f ca="1">TODAY()-5</f>
-        <v>45596</v>
+        <v>45604</v>
       </c>
       <c r="J6" s="25">
         <f ca="1">TODAY()+5</f>
-        <v>45606</v>
+        <v>45614</v>
       </c>
       <c r="K6" s="18">
         <v>6</v>
@@ -1748,11 +1889,11 @@
       </c>
       <c r="E7" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45609</v>
       </c>
       <c r="F7" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45626</v>
       </c>
       <c r="G7" s="18">
         <v>50</v>
@@ -1763,11 +1904,11 @@
       </c>
       <c r="I7" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45609</v>
       </c>
       <c r="J7" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45626</v>
       </c>
       <c r="K7" s="18">
         <v>4</v>
@@ -1794,11 +1935,11 @@
       </c>
       <c r="E8" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45609</v>
       </c>
       <c r="F8" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45626</v>
       </c>
       <c r="G8" s="18">
         <v>15</v>
@@ -1809,11 +1950,11 @@
       </c>
       <c r="I8" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45609</v>
       </c>
       <c r="J8" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45626</v>
       </c>
       <c r="K8" s="18">
         <v>1</v>
@@ -1840,11 +1981,11 @@
       </c>
       <c r="E9" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45609</v>
       </c>
       <c r="F9" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45626</v>
       </c>
       <c r="G9" s="18">
         <v>10</v>
@@ -1855,11 +1996,11 @@
       </c>
       <c r="I9" s="25">
         <f ca="1">TODAY()</f>
-        <v>45601</v>
+        <v>45609</v>
       </c>
       <c r="J9" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45626</v>
       </c>
       <c r="K9" s="18">
         <v>1</v>
@@ -1886,11 +2027,11 @@
       </c>
       <c r="E10" s="25">
         <f ca="1">TODAY()+3</f>
-        <v>45604</v>
+        <v>45612</v>
       </c>
       <c r="F10" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45626</v>
       </c>
       <c r="G10" s="18">
         <v>5</v>
@@ -1901,11 +2042,11 @@
       </c>
       <c r="I10" s="25">
         <f ca="1">TODAY()+3</f>
-        <v>45604</v>
+        <v>45612</v>
       </c>
       <c r="J10" s="25">
         <f ca="1">TODAY()+17</f>
-        <v>45618</v>
+        <v>45626</v>
       </c>
       <c r="K10" s="18">
         <v>6</v>
@@ -1996,21 +2137,22 @@
   <pageSetup fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <headerFooter differentFirst="1"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C52F64F2-A0CB-432E-B537-8AB164D6506B}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C52F64F2-A0CB-432E-B537-8AB164D6506B}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="13.5" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" style="27" customWidth="1"/>
-    <col min="2" max="2" width="20.0703125" style="27" customWidth="1"/>
-    <col min="3" max="3" width="16.7109375" style="27" customWidth="1"/>
-    <col min="4" max="16384" width="8.7109375" style="27"/>
+    <col min="1" max="1" width="12.7265625" style="27" customWidth="1"/>
+    <col min="2" max="2" width="20.08984375" style="27" customWidth="1"/>
+    <col min="3" max="3" width="16.7265625" style="27" customWidth="1"/>
+    <col min="4" max="16384" width="8.7265625" style="27"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2045,11 +2187,12 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2">
     <tabColor theme="7" tint="0.59999389629810485"/>
     <pageSetUpPr fitToPage="1"/>
@@ -2057,9 +2200,9 @@
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" style="12" customWidth="1"/>
-    <col min="2" max="3" width="18.42578125" style="23" customWidth="1"/>
-    <col min="4" max="4" width="6.7109375" style="13" customWidth="1"/>
+    <col min="1" max="1" width="6.7265625" style="12" customWidth="1"/>
+    <col min="2" max="3" width="18.453125" style="23" customWidth="1"/>
+    <col min="4" max="4" width="6.7265625" style="13" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
@@ -2069,7 +2212,7 @@
       <c r="C1" s="12"/>
       <c r="D1" s="12"/>
     </row>
-    <row r="2" spans="1:4" customFormat="1" ht="80.150000000000006" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" customFormat="1" ht="80.099999999999994" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="12"/>
       <c r="B2" s="16" t="s">
         <v>4</v>
@@ -2083,7 +2226,7 @@
       <c r="C3" s="13"/>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4" customFormat="1" ht="62.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" customFormat="1" ht="62.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="14"/>
       <c r="B4" s="22" t="s">
         <v>5</v>
@@ -2168,30 +2311,20 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup fitToHeight="0" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
   <tableParts count="1">
-    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Url xsi:nil="true"/>
-      <Description xsi:nil="true"/>
-    </Image>
-    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
-    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </ImageTagsTaxHTField>
-    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
-    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2507,22 +2640,29 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <Image xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Url xsi:nil="true"/>
+      <Description xsi:nil="true"/>
+    </Image>
+    <Status xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">Not started</Status>
+    <Background xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">false</Background>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <ImageTagsTaxHTField xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </ImageTagsTaxHTField>
+    <TaxCatchAll xmlns="230e9df3-be65-4c73-a93b-d1236ebd677e" xsi:nil="true"/>
+    <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9066C173-72E5-4455-ACFB-9A7596D30A2B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{648F31BC-5AA3-42BF-80F4-A797E59C4FBD}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
-    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2549,9 +2689,13 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{648F31BC-5AA3-42BF-80F4-A797E59C4FBD}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9066C173-72E5-4455-ACFB-9A7596D30A2B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5"/>
+    <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>